<commit_message>
2023.11.14 Comentado señales y esquema latex modelo
</commit_message>
<xml_diff>
--- a/DIA A DIA/DIARIO.xlsx
+++ b/DIA A DIA/DIARIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjime\Documents\ESTUDIOS\GRADO MATEMATICAS\4-CUARTO\TFG\GITHUB\DIA A DIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE89E39A-4442-42B0-B5ED-F010B59F4D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55D0145-3BC9-4D2E-8164-26D86E6B3B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve"> He instalado librerias y he añadido su directorio a PATH, al igual  pip install numpy pandas seaborn matplotlib tensorflow scikit-learn</t>
   </si>
@@ -69,7 +69,28 @@
     <t>Documentar el codigo de traffic sign entendiendo TODO</t>
   </si>
   <si>
-    <t>Probar con varias señales</t>
+    <t>02/10/2023 - 09/10/2023</t>
+  </si>
+  <si>
+    <t>Leer teoría a cerca de las redes neuronales de los apuntes de GCOM y TFG wuolah</t>
+  </si>
+  <si>
+    <t>Leer articulo de Cybersecurity NN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primera red neuronal en python </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red neuronal de XOR y predecir direccion coche </t>
+  </si>
+  <si>
+    <t>Crear documento de LaTeX, con portada y comentarios con citas sobre los libros/articulos leidos</t>
+  </si>
+  <si>
+    <t>Guardar ambos modelos con 20 epochs cada uno y guardad en el documento LaTeX lo que aparece por pantalla de cada modelo</t>
+  </si>
+  <si>
+    <t>Probar con algunos ejemplos.</t>
   </si>
 </sst>
 </file>
@@ -105,15 +126,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,10 +412,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B22"/>
+  <dimension ref="A2:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" style="1" customWidth="1"/>
     <col min="2" max="2" width="137.26953125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -418,8 +436,37 @@
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2"/>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
@@ -498,16 +545,23 @@
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A14:A18"/>
     <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A21:A23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
2023.11.17 Traffic sign OK
</commit_message>
<xml_diff>
--- a/DIA A DIA/DIARIO.xlsx
+++ b/DIA A DIA/DIARIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjime\Documents\ESTUDIOS\GRADO MATEMATICAS\4-CUARTO\TFG\GITHUB\DIA A DIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55D0145-3BC9-4D2E-8164-26D86E6B3B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEC341F-4595-4B3B-9905-796A6D60FE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve"> He instalado librerias y he añadido su directorio a PATH, al igual  pip install numpy pandas seaborn matplotlib tensorflow scikit-learn</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Escribir mi dia a dia de estas semanas atrás.</t>
   </si>
   <si>
-    <t>He estructurado mi codigo en funciones y he añadido algguna pagina web sobre los tipos de CNN, ademas de leer esa parte en el libro Aprendizaje profundo Cap 4</t>
-  </si>
-  <si>
     <t>Al comprobar con algunos numeros, los que estan de color blanco y fondo negro, funcionan. Los otros, fallan.</t>
   </si>
   <si>
@@ -91,14 +88,93 @@
   </si>
   <si>
     <t>Probar con algunos ejemplos.</t>
+  </si>
+  <si>
+    <t>Hemos eliminado el try, except a la hora de cargar los datos.</t>
+  </si>
+  <si>
+    <t>He estructurado mi codigo en funciones y he añadido algguna pagina web sobre los tipos de CNN, ademas de leer esa parte en el libro 
+Aprendizaje profundo Cap 4</t>
+  </si>
+  <si>
+    <t>Me he dado cuenta de como hacer los scrips mejor. Todo en funciones, nada de main. Hago una funcion que me cargue el modelo y en el 
+mismo script, otra funcion con los casos de prueba con dato de entrada el nombre de la imagen.</t>
+  </si>
+  <si>
+    <t>En la CNN de MNIST, me reconoce todos los numeros excepto algun ejemplo como el numero8.jpg que me predice un 5 pero podría serlo 
+perfectamente. Además, los numero que se salen del patron fondo negro y numero en blanco, no está asegurada su predicción correcta 
+como es el caso de numero6.png y numero0.png que tienen fondo oscuro y numero en oscuro.</t>
+  </si>
+  <si>
+    <t>Por lo general MNIST esta muy correcta.</t>
+  </si>
+  <si>
+    <t>semana 22 noviembre</t>
+  </si>
+  <si>
+    <t>Resolver el problema de las señales de trafico.</t>
+  </si>
+  <si>
+    <t>A ver si puedo solucionar el problema de los digitos con colores raros</t>
+  </si>
+  <si>
+    <t>Elegir del review, los ataques favoritos para empezar a abordarlos. Escogeré 3 o 4 que tengan diferentes ML methods</t>
+  </si>
+  <si>
+    <t>Guardar los graficos de mis redes</t>
+  </si>
+  <si>
+    <t>Escribir cada codigo de MNIST y TRAFFIC SIGN con mis palabras para ver cuanto he aprendido</t>
+  </si>
+  <si>
+    <t>plt.savefig(nombre) guardar una grafica o figura</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Me dan error la mayoria de las imágenes de señales de trafico. Vamos a ir depurando funcion a funcion a ver si a la hora de cargar los datos no se solapa bien la etiqueta con la imagen. Vamos a mostrar varios ejemplos de prueba que me digan si esta bien. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>He probado generando imagenes aleatorias pero he visto que no era muy eficiente ese metodo entonces he creado un grafico con la cantidad
+de imagenes por cada etiqueta y coincide con el numero de imagenes que me he descargado de cada clase. Ese no es el error.</t>
+    </r>
+  </si>
+  <si>
+    <t>ABRIR PYTHON EN TERMINAL
+PS C:\Users\pjime\Documents\ESTUDIOS\GRADO MATEMATICAS\4-CUARTO\TFG\GITHUB\CODIGOS\Reconocimiento de señales&gt; &amp; C:/Users/pjime/AppData/Local/Microsoft/WindowsApps/python3.9.exe
+C:/Users/pjime/AppData/Local/Microsoft/WindowsApps/python3.9.exe</t>
+  </si>
+  <si>
+    <t>He creado la matriz de confusiony todo correcto, he creado un grafico con la cantidad de imágenes de cada tipo y todo correcto(coincide con
+el numero de imágenes de cada clase guardadas en mis archivos) y por ultimo he generado imágenes aleatorias de las que estaban mal 
+en la matriz de confusion</t>
+  </si>
+  <si>
+    <t>He descubierto el error de mi codigo, en que en el modelo no normalizo y en mi prediccion si.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -126,9 +202,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -412,156 +500,239 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B23"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="137.26953125" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="119.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:2" ht="87" x14ac:dyDescent="0.35">
+      <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="6"/>
+      <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="6"/>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="6"/>
+      <c r="B8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="6"/>
+      <c r="B10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="6"/>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="6">
+        <v>45240</v>
+      </c>
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="6"/>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="6"/>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="6">
+        <v>45242</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="6"/>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="6"/>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="6"/>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="6"/>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="6">
+        <v>45243</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="6"/>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="6">
+        <v>45244</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="6"/>
+      <c r="B23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="2">
-        <v>45240</v>
-      </c>
-      <c r="B11" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
-      <c r="B12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="2"/>
-      <c r="B13" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="2">
-        <v>45242</v>
-      </c>
-      <c r="B14" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
-      <c r="B15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="2"/>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="2"/>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="B18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="2">
-        <v>45243</v>
-      </c>
-      <c r="B19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="2">
-        <v>45244</v>
-      </c>
-      <c r="B21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="6"/>
+      <c r="B24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="2"/>
-      <c r="B23" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="6">
+        <v>45245</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="6"/>
+      <c r="B26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="6"/>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="6"/>
+      <c r="B28" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="6"/>
+      <c r="B29" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="30" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="6"/>
+      <c r="B30" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>45246</v>
+      </c>
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B40" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="B43" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A21:A23"/>
+  <mergeCells count="7">
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A30"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A7:A11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
2023.11.28 Primeros pasos Malware detection
</commit_message>
<xml_diff>
--- a/DIA A DIA/DIARIO.xlsx
+++ b/DIA A DIA/DIARIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjime\Documents\ESTUDIOS\GRADO MATEMATICAS\4-CUARTO\TFG\GITHUB\DIA A DIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEC341F-4595-4B3B-9905-796A6D60FE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6E12E3-7552-4CF5-86A8-6CCC224D21A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve"> He instalado librerias y he añadido su directorio a PATH, al igual  pip install numpy pandas seaborn matplotlib tensorflow scikit-learn</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>Escribir mi dia a dia de estas semanas atrás.</t>
   </si>
   <si>
     <t>Al comprobar con algunos numeros, los que estan de color blanco y fondo negro, funcionan. Los otros, fallan.</t>
@@ -107,18 +104,6 @@
   </si>
   <si>
     <t>Por lo general MNIST esta muy correcta.</t>
-  </si>
-  <si>
-    <t>semana 22 noviembre</t>
-  </si>
-  <si>
-    <t>Resolver el problema de las señales de trafico.</t>
-  </si>
-  <si>
-    <t>A ver si puedo solucionar el problema de los digitos con colores raros</t>
-  </si>
-  <si>
-    <t>Elegir del review, los ataques favoritos para empezar a abordarlos. Escogeré 3 o 4 que tengan diferentes ML methods</t>
   </si>
   <si>
     <t>Guardar los graficos de mis redes</t>
@@ -159,6 +144,18 @@
   </si>
   <si>
     <t>He descubierto el error de mi codigo, en que en el modelo no normalizo y en mi prediccion si.</t>
+  </si>
+  <si>
+    <t>Nombre de los ficheros buenos : predicDigitosMNIST y trafficSign</t>
+  </si>
+  <si>
+    <t>Arreglado tema colores MNIST</t>
+  </si>
+  <si>
+    <t>Leer 4 articulos de malware asi por encima para entender sobre que va</t>
+  </si>
+  <si>
+    <t>Ver que tipo de datos hay y que incluyen el malware detection. Ver si se puede amoldar el mismo data para diferentes tipos de redes neuronales</t>
   </si>
 </sst>
 </file>
@@ -500,24 +497,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.54296875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="119.6328125" customWidth="1"/>
+    <col min="2" max="2" width="120.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -529,210 +523,238 @@
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
       <c r="B5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="6"/>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="6"/>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
         <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="6"/>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="6"/>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="6">
-        <v>45240</v>
-      </c>
-      <c r="B12" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="6"/>
-      <c r="B13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="6"/>
-      <c r="B14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="6">
-        <v>45242</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="6"/>
       <c r="B16" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="6"/>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="6"/>
       <c r="B18" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="6"/>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
-        <v>45243</v>
+        <v>45240</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="6"/>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="6">
-        <v>45244</v>
-      </c>
+      <c r="A22" s="6"/>
       <c r="B22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="6"/>
-      <c r="B23" t="s">
-        <v>19</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="6">
+        <v>45242</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="6"/>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="6">
-        <v>45245</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="6"/>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
-      <c r="B26" s="1" t="s">
-        <v>24</v>
+      <c r="B26" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="6"/>
       <c r="B27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="6"/>
-      <c r="B28" s="4" t="s">
-        <v>33</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="6">
+        <v>45243</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="6"/>
       <c r="B29" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="6"/>
-      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="6">
+        <v>45244</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="6"/>
+      <c r="B31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="6"/>
+      <c r="B32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="6">
+        <v>45245</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="6"/>
+      <c r="B34" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="6"/>
+      <c r="B35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="6"/>
+      <c r="B36" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="6"/>
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="6"/>
+      <c r="B38" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="6">
+        <v>45246</v>
+      </c>
+      <c r="B39" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="6"/>
+      <c r="B40" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="6"/>
+      <c r="B41" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="3">
+        <v>45259</v>
+      </c>
+      <c r="B49" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="3">
-        <v>45246</v>
-      </c>
-      <c r="B31" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B39" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B40" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B41" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B42" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="B43" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A25:A30"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A3:A5"/>
+  <mergeCells count="8">
     <mergeCell ref="A15:A19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A23:A27"/>
+    <mergeCell ref="A28:A29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>